<commit_message>
chore(examples): update example Excel files with new versions
</commit_message>
<xml_diff>
--- a/src/modules/excel/examples/data/table.xlsx
+++ b/src/modules/excel/examples/data/table.xlsx
@@ -484,7 +484,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="3">
-        <v>46144</v>
+        <v>46176</v>
       </c>
       <c r="B2" s="1">
         <v>0</v>
@@ -495,7 +495,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="3">
-        <v>46144.001000000004</v>
+        <v>46176.001000000004</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
@@ -506,7 +506,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="3">
-        <v>46144.002</v>
+        <v>46176.002</v>
       </c>
       <c r="B4" s="1">
         <v>2</v>
@@ -517,7 +517,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="3">
-        <v>46144.003</v>
+        <v>46176.003</v>
       </c>
       <c r="B5" s="1">
         <v>3</v>
@@ -528,7 +528,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="3">
-        <v>46144.004</v>
+        <v>46176.004</v>
       </c>
       <c r="B6" s="1">
         <v>4</v>
@@ -539,7 +539,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="3">
-        <v>46144.005000000005</v>
+        <v>46176.005000000005</v>
       </c>
       <c r="B7" s="1">
         <v>5</v>
@@ -550,7 +550,7 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="3">
-        <v>46144.006</v>
+        <v>46176.006</v>
       </c>
       <c r="B8" s="1">
         <v>6</v>
@@ -561,7 +561,7 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="3">
-        <v>46144.007</v>
+        <v>46176.007</v>
       </c>
       <c r="B9" s="1">
         <v>7</v>
@@ -572,7 +572,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="3">
-        <v>46144.008</v>
+        <v>46176.008</v>
       </c>
       <c r="B10" s="1">
         <v>8</v>
@@ -583,7 +583,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="3">
-        <v>46144.009</v>
+        <v>46176.009</v>
       </c>
       <c r="B11" s="1">
         <v>9</v>
@@ -594,7 +594,7 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="3">
-        <v>46144.009999999995</v>
+        <v>46176.009999999995</v>
       </c>
       <c r="B12" s="1">
         <v>10</v>
@@ -605,7 +605,7 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="3">
-        <v>46144.011</v>
+        <v>46176.011</v>
       </c>
       <c r="B13" s="1">
         <v>11</v>
@@ -616,7 +616,7 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="3">
-        <v>46144.012</v>
+        <v>46176.012</v>
       </c>
       <c r="B14" s="1">
         <v>12</v>

</xml_diff>